<commit_message>
Implement k6 API load testing pipeline and update E2E summaries
</commit_message>
<xml_diff>
--- a/automation/reports/excel/Execution_Summary.xlsx
+++ b/automation/reports/excel/Execution_Summary.xlsx
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24T06:54:04.206Z</t>
+    <t>2026-06-24T06:58:41.248Z</t>
   </si>
   <si>
     <t>Total Cases</t>
@@ -475,7 +475,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>504</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -483,7 +483,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove Appium server local dependency in package.json and update test reports
</commit_message>
<xml_diff>
--- a/automation/reports/excel/Execution_Summary.xlsx
+++ b/automation/reports/excel/Execution_Summary.xlsx
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24T06:58:41.248Z</t>
+    <t>2026-06-24T07:10:41.254Z</t>
   </si>
   <si>
     <t>Total Cases</t>
@@ -475,7 +475,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>496</v>
+        <v>505</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -483,7 +483,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update k6 configuration to 100 VUs x 1 Min and refresh E2E dashboards
</commit_message>
<xml_diff>
--- a/automation/reports/excel/Execution_Summary.xlsx
+++ b/automation/reports/excel/Execution_Summary.xlsx
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24T07:10:41.254Z</t>
+    <t>2026-06-24T07:38:12.343Z</t>
   </si>
   <si>
     <t>Total Cases</t>
@@ -475,7 +475,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>505</v>
+        <v>498</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -483,7 +483,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Populate 300 load test cases inside GHA expandable summary detail block
</commit_message>
<xml_diff>
--- a/automation/reports/excel/Execution_Summary.xlsx
+++ b/automation/reports/excel/Execution_Summary.xlsx
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24T07:38:12.343Z</t>
+    <t>2026-06-24T07:45:40.821Z</t>
   </si>
   <si>
     <t>Total Cases</t>
@@ -475,7 +475,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -483,7 +483,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>